<commit_message>
vault backup: 2026-07-22 18:12:20
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/软件概要设计-模块功能拆分-v2.xlsx
+++ b/公司项目/认知行动/文档/软件概要设计-模块功能拆分-v2.xlsx
@@ -4691,7 +4691,7 @@
         <x:v>M-SWM-07</x:v>
       </x:c>
       <x:c r="E36" t="str">
-        <x:v>按账号与画像自动生成提示词（提示词自动生成引擎）</x:v>
+        <x:v>对话编写提示词（对话编写引擎）</x:v>
       </x:c>
       <x:c r="F36" t="str">
         <x:v>R-SWM-005</x:v>
@@ -4763,28 +4763,28 @@
       </x:c>
     </x:row>
     <x:row r="41" spans="1:7" ht="90">
-      <x:c r="D41" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="E41" t="s">
-        <x:v>169</x:v>
-      </x:c>
-      <x:c r="F41" t="s">
-        <x:v>170</x:v>
+      <x:c r="D41" t="str">
+        <x:v>M-OCC-02</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>目标关联网络（目标关系图谱）</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>R-OCC-001(图结构)</x:v>
       </x:c>
       <x:c r="G41" s="8" t="s">
         <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:7" ht="54">
-      <x:c r="D42" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="E42" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="F42" t="s">
-        <x:v>174</x:v>
+      <x:c r="D42" t="str">
+        <x:v>M-OCC-03</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>数据分析与情报（情报分析大脑）</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>R-OCC-002~005</x:v>
       </x:c>
       <x:c r="G42" s="8" t="s">
         <x:v>175</x:v>
@@ -9104,8 +9104,8 @@
       <x:c r="B28" s="4" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="C28" s="5" t="s">
-        <x:v>148</x:v>
+      <x:c r="C28" s="5" t="str">
+        <x:v>对话编写提示词（对话编写引擎）</x:v>
       </x:c>
       <x:c r="D28" s="5" t="s">
         <x:v>149</x:v>
@@ -9570,8 +9570,8 @@
       <x:c r="D7" s="7" t="s">
         <x:v>857</x:v>
       </x:c>
-      <x:c r="E7" s="7" t="s">
-        <x:v>871</x:v>
+      <x:c r="E7" s="7" t="str">
+        <x:v>识别过程综合事件主体/传播源头与链路/事件群体账号传播画像/干预切入点与薄弱点，形成完整目标档案；融合本子系统数据分析与情报（M-OCC-03）的产出。</x:v>
       </x:c>
       <x:c r="F7" s="7" t="s">
         <x:v>872</x:v>
@@ -9579,8 +9579,8 @@
       <x:c r="G7" s="7" t="s">
         <x:v>860</x:v>
       </x:c>
-      <x:c r="H7" s="7" t="s">
-        <x:v>873</x:v>
+      <x:c r="H7" s="7" t="str">
+        <x:v>依赖 OCC 分析(M-OCC-03)/IRS</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:8" ht="27">
@@ -9609,212 +9609,212 @@
         <x:v>220</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" spans="1:8" ht="121.5">
+    <x:row r="9" spans="1:8" ht="54">
       <x:c r="A9" s="4" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="B9" s="4" t="s">
-        <x:v>168</x:v>
+      <x:c r="B9" s="4" t="str">
+        <x:v>M-OCC-02</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>169</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="D9" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="E9" s="5" t="s">
-        <x:v>171</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="F9" s="5" t="s">
-        <x:v>878</x:v>
+        <x:v>907</x:v>
       </x:c>
       <x:c r="G9" s="5" t="s">
-        <x:v>879</x:v>
+        <x:v>908</x:v>
       </x:c>
       <x:c r="H9" s="5" t="s">
-        <x:v>880</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:8" ht="27">
+        <x:v>909</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:8">
       <x:c r="A10" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="B10" s="6" t="s">
-        <x:v>881</x:v>
+      <x:c r="B10" s="6" t="str">
+        <x:v>F-OCC-02-01</x:v>
       </x:c>
       <x:c r="C10" s="7" t="s">
-        <x:v>882</x:v>
+        <x:v>911</x:v>
       </x:c>
       <x:c r="D10" s="7" t="s">
-        <x:v>883</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="E10" s="7" t="s">
-        <x:v>884</x:v>
+        <x:v>912</x:v>
       </x:c>
       <x:c r="F10" s="7" t="s">
-        <x:v>885</x:v>
+        <x:v>913</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>886</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="H10" s="7" t="s">
-        <x:v>887</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:8" ht="27">
+        <x:v>220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:8">
       <x:c r="A11" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="B11" s="6" t="s">
-        <x:v>888</x:v>
+      <x:c r="B11" s="6" t="str">
+        <x:v>F-OCC-02-02</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
-        <x:v>889</x:v>
+        <x:v>915</x:v>
       </x:c>
       <x:c r="D11" s="7" t="s">
-        <x:v>890</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="E11" s="7" t="s">
-        <x:v>891</x:v>
+        <x:v>916</x:v>
       </x:c>
       <x:c r="F11" s="7" t="s">
-        <x:v>892</x:v>
+        <x:v>917</x:v>
       </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>893</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="H11" s="7" t="s">
         <x:v>220</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" spans="1:8" ht="27">
-      <x:c r="A12" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="s">
-        <x:v>894</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
+    <x:row r="12" spans="1:8" ht="121.5">
+      <x:c r="A12" s="4" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>M-OCC-03</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="s">
+        <x:v>878</x:v>
+      </x:c>
+      <x:c r="G12" s="5" t="s">
+        <x:v>879</x:v>
+      </x:c>
+      <x:c r="H12" s="5" t="s">
+        <x:v>880</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:8" ht="27">
+      <x:c r="A13" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>F-OCC-03-01</x:v>
+      </x:c>
+      <x:c r="C13" s="7" t="s">
+        <x:v>882</x:v>
+      </x:c>
+      <x:c r="D13" s="7" t="s">
+        <x:v>883</x:v>
+      </x:c>
+      <x:c r="E13" s="7" t="s">
+        <x:v>884</x:v>
+      </x:c>
+      <x:c r="F13" s="7" t="s">
+        <x:v>885</x:v>
+      </x:c>
+      <x:c r="G13" s="7" t="s">
+        <x:v>886</x:v>
+      </x:c>
+      <x:c r="H13" s="7" t="s">
+        <x:v>887</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:8" ht="27">
+      <x:c r="A14" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>F-OCC-03-02</x:v>
+      </x:c>
+      <x:c r="C14" s="7" t="s">
+        <x:v>889</x:v>
+      </x:c>
+      <x:c r="D14" s="7" t="s">
+        <x:v>890</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="s">
+        <x:v>891</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="s">
+        <x:v>892</x:v>
+      </x:c>
+      <x:c r="G14" s="7" t="s">
+        <x:v>893</x:v>
+      </x:c>
+      <x:c r="H14" s="7" t="s">
+        <x:v>220</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:8" ht="27">
+      <x:c r="A15" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>F-OCC-03-03</x:v>
+      </x:c>
+      <x:c r="C15" s="7" t="s">
         <x:v>895</x:v>
       </x:c>
-      <x:c r="D12" s="7" t="s">
+      <x:c r="D15" s="7" t="s">
         <x:v>896</x:v>
       </x:c>
-      <x:c r="E12" s="7" t="s">
+      <x:c r="E15" s="7" t="s">
         <x:v>897</x:v>
       </x:c>
-      <x:c r="F12" s="7" t="s">
+      <x:c r="F15" s="7" t="s">
         <x:v>898</x:v>
       </x:c>
-      <x:c r="G12" s="7" t="s">
+      <x:c r="G15" s="7" t="s">
         <x:v>899</x:v>
-      </x:c>
-      <x:c r="H12" s="7" t="s">
-        <x:v>220</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:8" ht="40.5">
-      <x:c r="A13" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B13" s="6" t="s">
-        <x:v>900</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="s">
-        <x:v>901</x:v>
-      </x:c>
-      <x:c r="D13" s="7" t="s">
-        <x:v>902</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="s">
-        <x:v>903</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="s">
-        <x:v>904</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="s">
-        <x:v>905</x:v>
-      </x:c>
-      <x:c r="H13" s="7" t="s">
-        <x:v>906</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:8" ht="54">
-      <x:c r="A14" s="4" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="B14" s="4" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="E14" s="5" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="F14" s="5" t="s">
-        <x:v>907</x:v>
-      </x:c>
-      <x:c r="G14" s="5" t="s">
-        <x:v>908</x:v>
-      </x:c>
-      <x:c r="H14" s="5" t="s">
-        <x:v>909</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" spans="1:8">
-      <x:c r="A15" s="6" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="B15" s="6" t="s">
-        <x:v>910</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="s">
-        <x:v>911</x:v>
-      </x:c>
-      <x:c r="D15" s="7" t="s">
-        <x:v>857</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="s">
-        <x:v>912</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="s">
-        <x:v>913</x:v>
-      </x:c>
-      <x:c r="G15" s="7" t="s">
-        <x:v>860</x:v>
       </x:c>
       <x:c r="H15" s="7" t="s">
         <x:v>220</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" spans="1:8">
+    <x:row r="16" spans="1:8" ht="40.5">
       <x:c r="A16" s="6" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="B16" s="6" t="s">
-        <x:v>914</x:v>
+      <x:c r="B16" s="6" t="str">
+        <x:v>F-OCC-03-04</x:v>
       </x:c>
       <x:c r="C16" s="7" t="s">
-        <x:v>915</x:v>
+        <x:v>901</x:v>
       </x:c>
       <x:c r="D16" s="7" t="s">
-        <x:v>857</x:v>
+        <x:v>902</x:v>
       </x:c>
       <x:c r="E16" s="7" t="s">
-        <x:v>916</x:v>
+        <x:v>903</x:v>
       </x:c>
       <x:c r="F16" s="7" t="s">
-        <x:v>917</x:v>
+        <x:v>904</x:v>
       </x:c>
       <x:c r="G16" s="7" t="s">
-        <x:v>860</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="H16" s="7" t="s">
-        <x:v>220</x:v>
+        <x:v>906</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:8" ht="54">

</xml_diff>